<commit_message>
Auto update: scraping + analisis 2026-05-30 15:57 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,19 +417,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>topik</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -449,7 +437,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -457,7 +445,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -465,7 +453,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">
@@ -473,7 +461,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="n">

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-06-04 11:41 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>477</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>777</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>542</v>
+        <v>727</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>809</v>
+        <v>888</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>639</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-06-10 01:42 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>242</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>777</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>727</v>
+        <v>970</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>888</v>
+        <v>890</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>451</v>
+        <v>501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-06-14 01:34 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>323</v>
+        <v>870</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>448</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>970</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>890</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>501</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-06-22 01:39 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>870</v>
+        <v>885</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1060</v>
+        <v>632</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1081</v>
+        <v>955</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>292</v>
+        <v>515</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>419</v>
+        <v>746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-06-23 01:34 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>885</v>
+        <v>943</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>632</v>
+        <v>602</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>955</v>
+        <v>643</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>515</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>746</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-06-29 01:37 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>943</v>
+        <v>967</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>602</v>
+        <v>900</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>643</v>
+        <v>417</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1399</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>241</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-01 01:33 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>967</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>900</v>
+        <v>554</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>417</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1222</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>343</v>
+        <v>639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-02 01:36 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>554</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1283</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>639</v>
+        <v>610</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-16 01:24 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>567</v>
+        <v>619</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>409</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1299</v>
+        <v>647</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>610</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-18 01:20 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1073</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>619</v>
+        <v>854</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1239</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>647</v>
+        <v>459</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>384</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-24 01:28 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1077</v>
+        <v>736</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>854</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1161</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>459</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>414</v>
+        <v>482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-25 01:32 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>736</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>408</v>
+        <v>384</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1180</v>
+        <v>963</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1162</v>
+        <v>331</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>482</v>
+        <v>1210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-27 01:26 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1085</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>384</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>963</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>331</v>
+        <v>2378</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1210</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-07-28 01:31 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1172</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>306</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>152</v>
+        <v>543</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2378</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>113</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-03 01:26 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1150</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>120</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>543</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2103</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-05 01:31 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1167</v>
+        <v>928</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>259</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>2313</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>185</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>205</v>
+        <v>2429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-06 01:27 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>928</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>310</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>343</v>
+        <v>2209</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>120</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>2429</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-09 00:55 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1185</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>241</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>2209</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>288</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>212</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-10 00:59 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1199</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>193</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1156</v>
+        <v>501</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1404</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>228</v>
+        <v>1990</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-11 01:01 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1230</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>219</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>501</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>244</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1990</v>
+        <v>2206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-12 01:07 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1243</v>
+        <v>950</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>190</v>
+        <v>951</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>241</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>305</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>2206</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-13 01:06 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>950</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>951</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>277</v>
+        <v>469</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1606</v>
+        <v>563</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>408</v>
+        <v>1764</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-14 01:07 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1200</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>209</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>469</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>563</v>
+        <v>885</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1764</v>
+        <v>727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-15 00:48 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1165</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1169</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>270</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>885</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>727</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-16 00:45 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1266</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1061</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1495</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>252</v>
+        <v>2131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-19 00:46 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1283</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>210</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>320</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>287</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>2131</v>
+        <v>2355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-20 00:51 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1180</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>184</v>
+        <v>816</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>212</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>305</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>2355</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-27 05:46 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1264</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>816</v>
+        <v>514</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>247</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1690</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>228</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-30 02:34 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1414</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>514</v>
+        <v>502</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>174</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2166</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-08-31 02:35 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1406</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>502</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>183</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2176</v>
+        <v>815</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>145</v>
+        <v>879</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-09-03 02:24 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1428</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1072</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>220</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>815</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>879</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-09-10 02:10 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1354</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>215</v>
+        <v>674</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>2407</v>
+        <v>1755</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>201</v>
+        <v>388</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>295</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-09-12 02:16 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1590</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>674</v>
+        <v>946</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1755</v>
+        <v>790</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>388</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>222</v>
+        <v>1848</v>
       </c>
     </row>
   </sheetData>

</xml_diff>